<commit_message>
updated Link in BOM
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaure\Documents\GitHub\Bluetooth-and-Mioty-Localization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chand\Localisation in IOT git files\Git_hub_RP\Bluetooth-and-Mioty-Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40C7691-0827-4E95-97ED-D7C746445096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799AE4BC-AADB-4287-B8AE-C81CA0FCDB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -433,10 +433,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -459,10 +467,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -470,11 +479,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -754,16 +768,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" customWidth="1"/>
-    <col min="5" max="5" width="35.140625" customWidth="1"/>
-    <col min="6" max="6" width="138.140625" customWidth="1"/>
-    <col min="7" max="7" width="28.85546875" customWidth="1"/>
+    <col min="4" max="4" width="24.26953125" customWidth="1"/>
+    <col min="5" max="5" width="35.1796875" customWidth="1"/>
+    <col min="6" max="6" width="138.1796875" customWidth="1"/>
+    <col min="7" max="7" width="28.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -786,12 +800,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -805,12 +819,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -826,11 +840,11 @@
       <c r="E5" t="s">
         <v>125</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="4" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2</v>
       </c>
@@ -846,16 +860,16 @@
       <c r="E6" t="s">
         <v>122</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="4" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
@@ -871,16 +885,16 @@
       <c r="E8" t="s">
         <v>120</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -896,11 +910,11 @@
       <c r="E10" t="s">
         <v>110</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="4" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2</v>
       </c>
@@ -916,11 +930,11 @@
       <c r="E11" t="s">
         <v>106</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="4" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>3</v>
       </c>
@@ -936,11 +950,11 @@
       <c r="E12" t="s">
         <v>112</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>4</v>
       </c>
@@ -956,11 +970,11 @@
       <c r="E13" t="s">
         <v>112</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>5</v>
       </c>
@@ -976,11 +990,11 @@
       <c r="E14" t="s">
         <v>112</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>6</v>
       </c>
@@ -996,16 +1010,16 @@
       <c r="E15" t="s">
         <v>112</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1</v>
       </c>
@@ -1021,11 +1035,11 @@
       <c r="E17" t="s">
         <v>127</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1038,16 +1052,16 @@
       <c r="E18" t="s">
         <v>129</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="4" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1060,11 +1074,11 @@
       <c r="E20" t="s">
         <v>93</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2</v>
       </c>
@@ -1080,16 +1094,16 @@
       <c r="E21" t="s">
         <v>99</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1</v>
       </c>
@@ -1105,11 +1119,11 @@
       <c r="E23" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2</v>
       </c>
@@ -1125,11 +1139,11 @@
       <c r="E24" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>3</v>
       </c>
@@ -1145,11 +1159,11 @@
       <c r="E25" t="s">
         <v>31</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>4</v>
       </c>
@@ -1165,11 +1179,11 @@
       <c r="E26" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>5</v>
       </c>
@@ -1185,11 +1199,11 @@
       <c r="E27" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>6</v>
       </c>
@@ -1205,11 +1219,11 @@
       <c r="E28" t="s">
         <v>44</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>7</v>
       </c>
@@ -1225,11 +1239,11 @@
       <c r="E29" t="s">
         <v>39</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>8</v>
       </c>
@@ -1245,11 +1259,11 @@
       <c r="E30" t="s">
         <v>38</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>9</v>
       </c>
@@ -1265,11 +1279,11 @@
       <c r="E31" t="s">
         <v>48</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>10</v>
       </c>
@@ -1282,17 +1296,17 @@
       <c r="E32" t="s">
         <v>54</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>17</v>
       </c>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>1</v>
       </c>
@@ -1308,11 +1322,11 @@
       <c r="E34" t="s">
         <v>67</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1328,11 +1342,11 @@
       <c r="E35" t="s">
         <v>69</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3</v>
       </c>
@@ -1348,11 +1362,11 @@
       <c r="E36" t="s">
         <v>70</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>4</v>
       </c>
@@ -1368,11 +1382,11 @@
       <c r="E37" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>5</v>
       </c>
@@ -1388,11 +1402,11 @@
       <c r="E38" t="s">
         <v>83</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>6</v>
       </c>
@@ -1408,11 +1422,11 @@
       <c r="E39" t="s">
         <v>70</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>7</v>
       </c>
@@ -1428,11 +1442,11 @@
       <c r="E40" t="s">
         <v>77</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>8</v>
       </c>
@@ -1445,11 +1459,11 @@
       <c r="E41" t="s">
         <v>87</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>9</v>
       </c>
@@ -1460,7 +1474,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>10</v>
       </c>
@@ -1471,12 +1485,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>1</v>
       </c>
@@ -1492,11 +1506,45 @@
       <c r="E45" t="s">
         <v>92</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="4" t="s">
         <v>91</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F23" r:id="rId1" xr:uid="{D50FFC5A-821F-4C94-B04A-F406D35E99DC}"/>
+    <hyperlink ref="F20" r:id="rId2" xr:uid="{3206DE1E-5B1F-4613-AE54-DD3C9A177642}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{E06E345B-93C3-4FA7-935F-638068279AAA}"/>
+    <hyperlink ref="F6" r:id="rId4" xr:uid="{B5A236EB-917D-4615-83F0-A079BF0128A0}"/>
+    <hyperlink ref="F8" r:id="rId5" xr:uid="{848B4B6B-14A1-48B5-96A9-8F1107784A43}"/>
+    <hyperlink ref="F11" r:id="rId6" xr:uid="{F9107EB9-C9F2-4975-BB00-7BA16E1BD9B9}"/>
+    <hyperlink ref="F10" r:id="rId7" xr:uid="{C1C7415B-429D-491B-B931-EE38B7D918E5}"/>
+    <hyperlink ref="F12" r:id="rId8" xr:uid="{956B8FB4-224F-4E3B-92E7-CD01E96D4DAB}"/>
+    <hyperlink ref="F13" r:id="rId9" xr:uid="{4AC738DB-F9CA-435E-9BD3-136B300DF05D}"/>
+    <hyperlink ref="F14" r:id="rId10" xr:uid="{F56DB16A-7315-4DE4-A8FC-9739959F9F5B}"/>
+    <hyperlink ref="F15" r:id="rId11" xr:uid="{53C11F23-7475-46EB-8BBA-D8935F039069}"/>
+    <hyperlink ref="F17" r:id="rId12" xr:uid="{E90E8E5D-6049-4E64-A4CC-7A3C38EDE1BD}"/>
+    <hyperlink ref="F18" r:id="rId13" xr:uid="{BBE8552D-E013-4A5C-816F-6D9318AEA4EA}"/>
+    <hyperlink ref="F21" r:id="rId14" xr:uid="{CDE11C4C-F151-451A-B1BE-4E2FE821BEFA}"/>
+    <hyperlink ref="F24" r:id="rId15" xr:uid="{8E94842A-C938-4B1C-A463-8851C227BA1E}"/>
+    <hyperlink ref="F25" r:id="rId16" xr:uid="{6EF2DEF8-3A9E-4603-B943-6D14C205FA99}"/>
+    <hyperlink ref="F26" r:id="rId17" xr:uid="{2DCBF906-DF54-4368-BC71-B26C97E8F048}"/>
+    <hyperlink ref="F39" r:id="rId18" xr:uid="{44AD2C82-A23C-4467-930A-48D7D3770B50}"/>
+    <hyperlink ref="F30" r:id="rId19" xr:uid="{3D8C70F3-86D1-408F-B991-32BBA9AE0284}"/>
+    <hyperlink ref="F29" r:id="rId20" xr:uid="{B4530D85-708B-4214-B1E4-BAFC599C8674}"/>
+    <hyperlink ref="F27" r:id="rId21" xr:uid="{467D3286-50FF-4216-8937-835A6BA4C3A8}"/>
+    <hyperlink ref="F28" r:id="rId22" xr:uid="{283DFAF0-B027-460E-BEA3-E28DB7D75637}"/>
+    <hyperlink ref="F31" r:id="rId23" xr:uid="{217435C8-5FF7-4B86-B4E9-BFA135B39084}"/>
+    <hyperlink ref="F32" r:id="rId24" xr:uid="{F9702DF9-CC1B-42B0-96AD-216A11C735E3}"/>
+    <hyperlink ref="F34" r:id="rId25" xr:uid="{A27D8FF2-1762-470C-89EB-CA17719CDF2A}"/>
+    <hyperlink ref="F35" r:id="rId26" xr:uid="{CB456E9B-1680-41E5-A8F6-0AC98E1B2684}"/>
+    <hyperlink ref="F36" r:id="rId27" xr:uid="{84C8FBE4-112A-49FF-8A0D-F9CB3B1FE98A}"/>
+    <hyperlink ref="F37" r:id="rId28" xr:uid="{7AB50742-9609-4684-BB22-23FCC3D0AFAC}"/>
+    <hyperlink ref="F38" r:id="rId29" xr:uid="{CEB15CA5-20DF-48F1-A71E-97BE776E1A3A}"/>
+    <hyperlink ref="F40" r:id="rId30" xr:uid="{7DC9F4BF-0E00-4FE8-9952-52FD0B31FE2B}"/>
+    <hyperlink ref="F41" r:id="rId31" display="https://www.digikey.de/de/products/detail/te-connectivity-linx/CONMHF1-SMD-G-T/15293397?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20179951824&amp;gbraid=0AAAAADrbLlgcW0wDpxdB3QLoBqEJ77uUK&amp;gclid=Cj0KCQjw6bfHBhDNARIsAIGsqLjLl1jPmqBYngNawJjpDc2NL71_ijr013dRm_6SUY6Z-PSxDqZcU4AaAjl_EALw_wcB" xr:uid="{72808A11-5911-4A58-ADDF-A972CB0F47C2}"/>
+    <hyperlink ref="F45" r:id="rId32" xr:uid="{EBB4519B-B72F-4CC1-9062-C7A3B3B0DDF2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Schematic, BOM, Add Symbols and completed 3d view
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\OneDrive\Documents\FAU\BLE MIOTY MAIN\GAURAV SUPER KINGS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\OneDrive\Documents\FAU\BLE MIOTY\Bluetooth-and-Mioty-Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD91BA4-0B67-4626-A41C-C0EAE2C38E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C572AAC5-5B0E-4727-93EF-8B244CFD2B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="770" windowWidth="25600" windowHeight="15230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="176">
   <si>
     <t>S. No.</t>
   </si>
@@ -544,6 +544,15 @@
   </si>
   <si>
     <t>C0402C105K8PACTU</t>
+  </si>
+  <si>
+    <t>C99</t>
+  </si>
+  <si>
+    <t>C24</t>
+  </si>
+  <si>
+    <t>U2</t>
   </si>
 </sst>
 </file>
@@ -923,17 +932,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G68"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="23.7265625" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="35.140625" customWidth="1"/>
-    <col min="6" max="6" width="148.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="35.1796875" customWidth="1"/>
+    <col min="6" max="6" width="148.81640625" customWidth="1"/>
+    <col min="7" max="7" width="28.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -956,12 +965,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -981,7 +990,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1001,12 +1010,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>1</v>
       </c>
@@ -1026,7 +1035,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>2</v>
       </c>
@@ -1046,12 +1055,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -1071,12 +1080,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>1</v>
       </c>
@@ -1096,7 +1105,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>2</v>
       </c>
@@ -1116,7 +1125,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>3</v>
       </c>
@@ -1136,7 +1145,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>4</v>
       </c>
@@ -1156,7 +1165,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>5</v>
       </c>
@@ -1176,7 +1185,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>6</v>
       </c>
@@ -1196,12 +1205,12 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>1</v>
       </c>
@@ -1221,7 +1230,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>2</v>
       </c>
@@ -1241,17 +1250,17 @@
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>1</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>86</v>
+        <v>175</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>15</v>
@@ -1264,7 +1273,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>2</v>
       </c>
@@ -1284,7 +1293,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>3</v>
       </c>
@@ -1304,7 +1313,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>4</v>
       </c>
@@ -1324,7 +1333,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>5</v>
       </c>
@@ -1344,7 +1353,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>6</v>
       </c>
@@ -1364,7 +1373,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>7</v>
       </c>
@@ -1384,7 +1393,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>8</v>
       </c>
@@ -1404,12 +1413,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
         <v>1</v>
       </c>
@@ -1429,7 +1438,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>2</v>
       </c>
@@ -1449,7 +1458,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>3</v>
       </c>
@@ -1469,7 +1478,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>4</v>
       </c>
@@ -1489,7 +1498,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>5</v>
       </c>
@@ -1509,7 +1518,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>6</v>
       </c>
@@ -1529,7 +1538,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>7</v>
       </c>
@@ -1549,7 +1558,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>8</v>
       </c>
@@ -1569,7 +1578,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>9</v>
       </c>
@@ -1589,7 +1598,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>10</v>
       </c>
@@ -1609,7 +1618,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>11</v>
       </c>
@@ -1627,7 +1636,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>17</v>
       </c>
@@ -1637,7 +1646,7 @@
       <c r="E41" s="2"/>
       <c r="F41" s="10"/>
     </row>
-    <row r="42" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>1</v>
       </c>
@@ -1657,7 +1666,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>2</v>
       </c>
@@ -1677,7 +1686,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>3</v>
       </c>
@@ -1697,7 +1706,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>4</v>
       </c>
@@ -1717,7 +1726,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>5</v>
       </c>
@@ -1737,7 +1746,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>6</v>
       </c>
@@ -1757,7 +1766,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>7</v>
       </c>
@@ -1773,7 +1782,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>8</v>
       </c>
@@ -1791,12 +1800,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>9</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>60</v>
@@ -1807,7 +1816,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>10</v>
       </c>
@@ -1823,17 +1832,17 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>1</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>79</v>
+        <v>173</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>80</v>
@@ -1848,12 +1857,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>1</v>
       </c>
@@ -1873,7 +1882,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>2</v>
       </c>
@@ -1893,7 +1902,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>3</v>
       </c>
@@ -1913,7 +1922,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>4</v>
       </c>
@@ -1933,7 +1942,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>5</v>
       </c>
@@ -1953,7 +1962,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>6</v>
       </c>
@@ -1973,12 +1982,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>1</v>
       </c>
@@ -1998,7 +2007,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>2</v>
       </c>
@@ -2018,7 +2027,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>3</v>
       </c>
@@ -2038,7 +2047,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>4</v>
       </c>
@@ -2058,7 +2067,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>5</v>
       </c>
@@ -2078,7 +2087,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>6</v>
       </c>
@@ -2098,7 +2107,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F68" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed tantal ref C33
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\OneDrive\Documents\FAU\BLE MIOTY\Bluetooth-and-Mioty-Localization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaure\Documents\GitHub\Bluetooth-and-Mioty-Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C572AAC5-5B0E-4727-93EF-8B244CFD2B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BF4F71-92FF-4D04-A689-F12224C4EC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -546,13 +546,13 @@
     <t>C0402C105K8PACTU</t>
   </si>
   <si>
-    <t>C99</t>
-  </si>
-  <si>
     <t>C24</t>
   </si>
   <si>
     <t>U2</t>
+  </si>
+  <si>
+    <t>C33</t>
   </si>
 </sst>
 </file>
@@ -932,17 +932,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="23.7265625" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
     <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="35.1796875" customWidth="1"/>
-    <col min="6" max="6" width="148.81640625" customWidth="1"/>
-    <col min="7" max="7" width="28.81640625" customWidth="1"/>
+    <col min="5" max="5" width="35.140625" customWidth="1"/>
+    <col min="6" max="6" width="148.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -965,12 +965,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -990,7 +990,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1010,12 +1010,12 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>1</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>2</v>
       </c>
@@ -1055,12 +1055,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>1</v>
       </c>
@@ -1080,12 +1080,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>1</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>2</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>3</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>4</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>5</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>6</v>
       </c>
@@ -1205,12 +1205,12 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>1</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>2</v>
       </c>
@@ -1250,17 +1250,17 @@
         <v>116</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>1</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>15</v>
@@ -1273,7 +1273,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>2</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>3</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>4</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>5</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>6</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>7</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>8</v>
       </c>
@@ -1413,12 +1413,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>1</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>2</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>3</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>4</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>5</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>6</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>7</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>8</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>9</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>10</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>11</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>17</v>
       </c>
@@ -1646,7 +1646,7 @@
       <c r="E41" s="2"/>
       <c r="F41" s="10"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>1</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>2</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>3</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>4</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>5</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>6</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>7</v>
       </c>
@@ -1782,7 +1782,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>8</v>
       </c>
@@ -1800,12 +1800,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>9</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>60</v>
@@ -1816,7 +1816,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>10</v>
       </c>
@@ -1832,17 +1832,17 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>1</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>80</v>
@@ -1857,12 +1857,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>1</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>2</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>3</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>4</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>5</v>
       </c>
@@ -1962,7 +1962,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>6</v>
       </c>
@@ -1982,12 +1982,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>1</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>2</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>3</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>4</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>5</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>6</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F68" s="1"/>
     </row>
   </sheetData>

</xml_diff>